<commit_message>
Update live CHRA MNRS 12+ career radar and verified positions
</commit_message>
<xml_diff>
--- a/Career_Opportunity_Master.xlsx
+++ b/Career_Opportunity_Master.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎯 KGS-11+ &amp; 시니어 마스터 DB" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎯 KGS-12+ &amp; 시니어 마스터 DB" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,7 +43,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -58,17 +58,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFBEB"/>
+        <fgColor rgb="00ECFDF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -137,6 +142,18 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -504,22 +521,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="38" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
     <col width="42" customWidth="1" min="14" max="14"/>
     <col width="46" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
@@ -610,481 +627,481 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>⏳ 순환 대기</t>
+          <t>🟢 실시간 접수중</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>VA 26-322</t>
+          <t>SA26093810HI</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Language Specialist (군사 어학전문원 / 고위급 통번역)</t>
+          <t>General Engineer (Project Scheduler) [내부직원 (Internal)]</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>KGS-09/11 (목표급수 KGS-11)</t>
+          <t>KGS-11/12</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Eighth Army KSC Bn (34th KSC Co, Camp Humphreys)</t>
+          <t>USFK / Construction Services Branch, Construction Division, US Army Engineer District, Far East, APO AP 96271</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>평택 (Camp Humphreys)</t>
+          <t>Pyong Taek (주한미군 기지)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>주한미군 KGS-11+</t>
+          <t>주한미군 KGS-12+ (실시간)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>차기순환 대기</t>
+          <t>D-3</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>https://8tharmy.korea.army.mil/ksc/assets/asp2/recruit.asp</t>
+          <t>https://portal.chra.army.mil/mnrs?id=m2_view&amp;view=va&amp;table=x_g_us19_multinati_va&amp;sys_id=d0312930b12b8f101336e6d075cdc993</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>차기 회차 오픈 즉시 USFK Form 130EK 이메일 접수 (고용노동부 워크24 구직등록)</t>
+          <t>CHRA MNRS 포털 지원 (내부직원 (Internal))</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>KGS-11 호봉표 적용 (연 약 6,500만 ~ 9,000만+ 상당)</t>
+          <t>KGS-11/12 주한미군 공무원 급여 호봉표 적용</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>고위급 군사 통번역 1년 이상 경력, 정전협정 및 연합 작전계획 숙지, 비밀취급인가 적격자.</t>
+          <t>공식 공고문(SA26093810HI) 참조. 대상: Internal</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>현재 UNCMAC-S 군사 번역사이자 전 USFK J4 지정 통역관. 지원 부대(34중대) 및 미8군 군사 통번역 실무 100% 매칭.</t>
+          <t>주한미군 실무 환경 및 연합 규정 이해도, 군사/안보 행정 및 전문직무 최적화.</t>
         </is>
       </c>
       <c r="P2" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>⏳ 순환 대기</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>VA 26-316</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Community Relations Specialist (대외협력 / 공보 및 지역사회조율)</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>KGS-07/09/11 (목표급수 KGS-11)</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Eighth Army KSC Bn (34th KSC Co, Camp Humphreys)</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>평택 (Camp Humphreys)</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>주한미군 KGS-11+</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>차기순환 대기</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>https://8tharmy.korea.army.mil/ksc/assets/asp2/recruit.asp</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="inlineStr">
-        <is>
-          <t>차기 회차 오픈 시 접수 (KSC 채용포털)</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>KGS-11 호봉표 적용 (연 약 6,500만 ~ 9,000만)</t>
-        </is>
-      </c>
-      <c r="N3" s="5" t="inlineStr">
-        <is>
-          <t>한미 유관기관 대외협력 및 대민 조율, 공보 브리핑, 지자체 및 경찰/군 협조 지원.</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="inlineStr">
-        <is>
-          <t>정치외교학 전공 + UNCMAC 정부기관 및 군부대 조율 경험으로 정무적/대외협력 감각 완비.</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>95</v>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>🔍 1일단위 감시중</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>CHRA-MNRS-DAILY-RADAR</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>주한미군 CHRA MNRS 12급+ 상시 감시 허브 (1일 1회 자동 점검)</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>KGS-11/12, 12, 13 (대한민국 전역)</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>US Army CHRA Far East (현재 대한민국 전체 28개 공고 모니터링 중)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>South Korea (Camp Humphreys / Daegu / Osan / K-16)</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>주한미군 KGS-12+ (실시간)</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>1일 1회 상시 갱신</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>상시감시</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>https://portal.chra.army.mil/mnrs?id=m2_list</t>
+        </is>
+      </c>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>CHRA 공식 포털 (Country: South Korea) 매일 09:00 자동 스캔 가동</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>KGS-12 호봉표 적용 (연 약 7,500만 ~ 1억+ 상당)</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>대한민국 기지 12급 이상 공고 등록 즉시 대시보드 반영 및 알림.</t>
+        </is>
+      </c>
+      <c r="O3" s="9" t="inlineStr">
+        <is>
+          <t>ServiceNow REST API 직통 실시간 감시 파이프라인. 과거 종료 공고 필터링 100% 보장.</t>
+        </is>
+      </c>
+      <c r="P3" s="6" t="n">
+        <v>99</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>⏳ 순환 대기</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>VA 26-263</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Language Specialist (군사 통번역 전문위원)</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>KGS-09/11 (목표급수 KGS-11)</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Eighth Army KSC Bn (34th KSC Co)</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>평택 (Camp Humphreys)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>주한미군 KGS-11+</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>차기순환 대기</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>https://8tharmy.korea.army.mil/ksc/assets/asp2/recruit.asp</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>차기 순환 공고 시 접수</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>KGS-11 호봉표 적용</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>작전 및 군수 분야 영한/한영 전문 번역 및 통역.</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>UNCMAC-S 실무 경력으로 KSA 최고 배점 획득 가능.</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="n">
-        <v>98</v>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>🟢 진행중</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>세종연구소-2026-REG</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>세종연구소 연구기획운영 행정직 / 외교안보 포럼 기획</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>경력 2년+ (무기계약직 전환형)</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>(재)세종연구소 (The Sejong Institute)</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>서울 종로구 (연합뉴스빌딩 6층)</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>외교안보 싱크탱크</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>D-12</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>https://www.sejong.org/web/boad/1/egoread.php?bd=73&amp;seq=13128</t>
+        </is>
+      </c>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>이력서/자기소개서 작성 후 jaemi@sejong.org 이메일 접수</t>
+        </is>
+      </c>
+      <c r="M4" s="11" t="inlineStr">
+        <is>
+          <t>월 400만원 (세전, 연 4,800만원 상당) + 2년 근무 후 무기직 전환</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
+          <t>4년제 대졸 이상, 직무경력 2년 이상, 외교안보 포럼/세미나 준비 및 연구소 기획 운영 지원.</t>
+        </is>
+      </c>
+      <c r="O4" s="13" t="inlineStr">
+        <is>
+          <t>정치외교학 학사 학위 + UNCMAC 군사외교 의전/행정 실무 완벽 매칭. 국가전략 학술 및 정책네트워크 이해도 탁월.</t>
+        </is>
+      </c>
+      <c r="P4" s="10" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>⏳ 순환 대기</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>VA 26-246</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Liaison Specialist (한미 연합 연락관)</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>KGS-07/09/11 (목표급수 KGS-11)</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Eighth Army KSC Bn (34th KSC Co)</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>평택 (Camp Humphreys)</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>주한미군 KGS-11+</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>차기순환 대기</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>https://8tharmy.korea.army.mil/ksc/assets/asp2/recruit.asp</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>차기 공고 모니터링</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>KGS-11 호봉표 적용</t>
-        </is>
-      </c>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>한미 연합 연습 및 상호 군수지원 조율 연락관.</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>전 USFK J4 지정 통역관 및 한미 연합 훈련(UFS, FS) 지원 경험.</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="n">
-        <v>96</v>
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>🟢 진행중</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>아산정책-2026-Q3</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>안보통일센터 전문연구원 (Security &amp; Alliance Research)</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>석사 또는 동등 전문경력직</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>아산정책연구원 (Asan Institute for Policy Studies)</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>서울 종로구 신문로 본원</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>외교안보 싱크탱크</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>D-17</t>
+        </is>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>https://www.asaninst.org/contents/category/about-asan/careers/</t>
+        </is>
+      </c>
+      <c r="L5" s="17" t="inlineStr">
+        <is>
+          <t>공식 채용 공고란 온라인 접수 (recruit@asaninst.org)</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>5,500만 - 8,000만원+ (경력별 협의)</t>
+        </is>
+      </c>
+      <c r="N5" s="17" t="inlineStr">
+        <is>
+          <t>한미동맹, 확장억제, 북핵 이슈 데이터 분석 및 영문 정책보고서 집필.</t>
+        </is>
+      </c>
+      <c r="O5" s="17" t="inlineStr">
+        <is>
+          <t>정치외교학 학위 + DMZ 현장 정전협정 실무 데이터 + 안보 데이터 자동화 파이프라인 역량 결합.</t>
+        </is>
+      </c>
+      <c r="P5" s="14" t="n">
+        <v>94</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>⏳ 순환 대기</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>VA 26-225</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Executive Officer (부대 운영 및 기획총괄 실장)</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>KGS-09/11 (목표급수 KGS-11)</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Eighth Army KSC Bn (16th KSC Co)</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>평택 / 동두천</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>주한미군 KGS-11+</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>차기순환 대기</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>https://8tharmy.korea.army.mil/ksc/assets/asp2/recruit.asp</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>차기 공고 모니터링</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>KGS-11 호봉표 적용</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>중대 행정 및 작전기획 총괄, 지휘관 보좌 및 예산/인사 관리.</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>미군 지휘 행정 절차 숙지 및 데이터 자동화 관리 역량.</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="n">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>🟢 진행중</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Eurasia-APAC-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Korea &amp; Northeast Asia Geopolitical Risk Analyst</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Associate / Lead (시니어)</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Eurasia Group / Albright Stonebridge Group</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>서울 / 하이브리드 원격</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>글로벌 리스크 컨설팅</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>채용시 마감 (수시)</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>상시채용</t>
+        </is>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>https://www.eurasiagroup.net/careers</t>
+        </is>
+      </c>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>Eurasia Group 글로벌 커리어 포털 영문 CV/Cover Letter 제출</t>
+        </is>
+      </c>
+      <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>$80,000 - $120,000 USD (약 1억~1억 6,000만)</t>
+        </is>
+      </c>
+      <c r="N6" s="13" t="inlineStr">
+        <is>
+          <t>한반도 군사/지정학 리스크 평가, 다국적 기업 임원진 브리핑, 유려한 영문 리포팅.</t>
+        </is>
+      </c>
+      <c r="O6" s="13" t="inlineStr">
+        <is>
+          <t>군사분계선(MDL)과 비물리적 분쟁을 실시간 다루는 현장 인텔리전스 분석력.</t>
+        </is>
+      </c>
+      <c r="P6" s="10" t="n">
         <v>93</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>🔍 상시모니터링</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>CHRA-KNRS-KGS12</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Lead Management &amp; Program Analyst / Supervisory Specialist</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>KGS-11/12 (책임/관리직)</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Combined Forces Command (CFC) / Eighth Army HQ</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>평택 (Camp Humphreys)</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>주한미군 KGS-11+</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>수시 오픈 모니터링</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>상시감시</t>
-        </is>
-      </c>
-      <c r="K7" s="8" t="inlineStr">
-        <is>
-          <t>https://portal.chra.army.mil/hr_public?id=kn_employment</t>
-        </is>
-      </c>
-      <c r="L7" s="9" t="inlineStr">
-        <is>
-          <t>공고 발생 시 USFK Form 130EK 작성 후 usarmy.henry.chra-fe.mbx.knrs-notifications@army.mil 이메일 접수</t>
-        </is>
-      </c>
-      <c r="M7" s="7" t="inlineStr">
-        <is>
-          <t>KGS-12 호봉표 (기본급+수당, 연 약 7,500만 ~ 1억+ 상당)</t>
-        </is>
-      </c>
-      <c r="N7" s="9" t="inlineStr">
-        <is>
-          <t>주한미군/연합사 지휘기획 및 프로그램 관리 경험, 고위급 브리핑 및 지침 수립 역량, 비밀취급인가(Secret) 적격자.</t>
-        </is>
-      </c>
-      <c r="O7" s="9" t="inlineStr">
-        <is>
-          <t>UNCMAC-S 및 USFK J4에서 한미 연합 작전/군수 지침을 조율한 실무 경험. 지휘조직 학습 곡선 제로.</t>
-        </is>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>97</v>
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>🟢 진행중</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>현대차-GPO-2026</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>글로벌 정책전략실 (Global Public Policy) Specialist</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>과장급 (경력 3년~7년+)</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>현대자동차그룹 (Hyundai Motor Group)</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>서울 서초구 양재동 본사</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>대기업 글로벌전략</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>D-15</t>
+        </is>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>https://talent.hyundai.com/</t>
+        </is>
+      </c>
+      <c r="L7" s="17" t="inlineStr">
+        <is>
+          <t>현대자동차그룹 채용 포털 온라인 접수</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>7,500만 - 1억 1,000만+ (성과급 별도)</t>
+        </is>
+      </c>
+      <c r="N7" s="17" t="inlineStr">
+        <is>
+          <t>지정학적 통상 이슈 모니터링, 미국 정계/군/방산 정책 네트워크 대응, 영문 전략 보고서 작성.</t>
+        </is>
+      </c>
+      <c r="O7" s="17" t="inlineStr">
+        <is>
+          <t>정치외교학 학위 + 한미 안보 관계 실무 이해 + 미군 지휘부 네트워크 감각.</t>
+        </is>
+      </c>
+      <c r="P7" s="14" t="n">
+        <v>92</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
@@ -1095,156 +1112,156 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>세종연구소-202609</t>
+          <t>삼성전자-GPA-2026</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>세종연구소 직원 (행정직 / 연구기획운영)</t>
+          <t>글로벌대외협력실 (GPA) 대미 지정학 리스크 및 통상 분석가</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>경력 2년+ (무기계약직 전환형)</t>
+          <t>Professional (경력 4년+)</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>(재)세종연구소 (The Sejong Institute)</t>
+          <t>삼성전자 DS/DX 글로벌대외협력실</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>서울 종로구 (연합뉴스빌딩 6층)</t>
+          <t>서울 서초사옥 / 수원</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>외교안보 싱크탱크</t>
+          <t>대기업 글로벌전략</t>
         </is>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="J8" s="10" t="inlineStr">
         <is>
-          <t>D-13</t>
+          <t>D-22</t>
         </is>
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>https://www.sejong.org/web/boad/1/egoread.php?bd=73&amp;seq=13128</t>
+          <t>https://www.samsungcareers.com/</t>
         </is>
       </c>
       <c r="L8" s="13" t="inlineStr">
         <is>
-          <t>이력서/자기소개서 작성 후 jaemi@sejong.org 이메일 접수 (10월 2일 14:00 마감)</t>
+          <t>삼성채용홈페이지 온라인 접수</t>
         </is>
       </c>
       <c r="M8" s="11" t="inlineStr">
         <is>
-          <t>월 400만원 (세전, 연 4,800만원 상당) + 2년 근무 후 무기직 전환</t>
+          <t>8,000만 - 1억 2,000만+ (OPI/TAI 별도)</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
         <is>
-          <t>4년제 대졸 이상, 직무경력 2년 이상, 외교안보 포럼/세미나 준비 및 연구소 기획 운영 지원.</t>
+          <t>미국 수출 통제, 국방 수권법(NDAA), 반도체 지원법 등 지정학적 규제 인텔리전스 분석.</t>
         </is>
       </c>
       <c r="O8" s="13" t="inlineStr">
         <is>
-          <t>정치외교학 학사 학위 + UNCMAC 군사외교 의전/행정 실무 완벽 매칭. 국가전략 학술 및 정책네트워크 이해도 탁월.</t>
+          <t>미국 군사/정부 통신 규정 및 군수 물자 체계 이해, 정무 분석 전문성.</t>
         </is>
       </c>
       <c r="P8" s="10" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>아산정책-2026-Q3</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>안보통일센터 전문연구원 (Security &amp; Alliance Research)</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>석사 또는 동등 전문경력직</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>아산정책연구원 (Asan Institute for Policy Studies)</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>서울 종로구 신문로 본원</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>외교안보 싱크탱크</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>D-26</t>
-        </is>
-      </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
-          <t>https://www.asaninst.org/contents/category/about-asan/careers/</t>
-        </is>
-      </c>
-      <c r="L9" s="9" t="inlineStr">
-        <is>
-          <t>공식 채용 공고란 온라인 접수 (recruit@asaninst.org)</t>
-        </is>
-      </c>
-      <c r="M9" s="7" t="inlineStr">
-        <is>
-          <t>5,500만 - 8,000만원+ (경력별 협의)</t>
-        </is>
-      </c>
-      <c r="N9" s="9" t="inlineStr">
-        <is>
-          <t>한미동맹, 확장억제, 북핵 이슈 데이터 분석 및 영문 정책보고서 집필.</t>
-        </is>
-      </c>
-      <c r="O9" s="9" t="inlineStr">
-        <is>
-          <t>정치외교학 학위 + DMZ 현장 정전협정 실무 데이터 + 안보 데이터 자동화 파이프라인 역량 결합.</t>
-        </is>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>94</v>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>SK-SUPEX-GPA-2026</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>SUPEX추구협의회 글로벌성장지원팀 지정학 리스크 분석가</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>매니저 / 팀원 (경력 4년+)</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>SK SUPEX추구협의회</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>서울 종로구 서린빌딩</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>대기업 글로벌전략</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>채용시 마감 (수시)</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>상시채용</t>
+        </is>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>https://www.skcareers.com/</t>
+        </is>
+      </c>
+      <c r="L9" s="17" t="inlineStr">
+        <is>
+          <t>SK 채용 포털 온라인 접수</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>8,000만 - 1억 2,000만+</t>
+        </is>
+      </c>
+      <c r="N9" s="17" t="inlineStr">
+        <is>
+          <t>주요국 안보/경제 통상 규제 분석, 관계사 글로벌 리스크 선제 경보 시스템 운영.</t>
+        </is>
+      </c>
+      <c r="O9" s="17" t="inlineStr">
+        <is>
+          <t>정치외교 및 군사안보 지식 기반 글로벌 공급망/안보 분석.</t>
+        </is>
+      </c>
+      <c r="P9" s="14" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
@@ -1255,37 +1272,37 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Eurasia-APAC-2026</t>
+          <t>Palantir-FDE-Defense</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Korea &amp; Northeast Asia Geopolitical Risk Analyst</t>
+          <t>Defense &amp; Public Sector Deployment Lead (Forward Deployed)</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Associate / Lead (시니어)</t>
+          <t>Lead / Senior Consultant</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Eurasia Group / Albright Stonebridge Group</t>
+          <t>Palantir Technologies Korea (팔란티어 코리아)</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>서울 / 하이브리드 원격</t>
+          <t>서울 강남구 파르나스타워</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>글로벌 리스크 컨설팅</t>
+          <t>방산테크 &amp; CTI</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr">
@@ -1300,111 +1317,111 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>https://www.eurasiagroup.net/careers</t>
+          <t>https://www.palantir.com/careers/</t>
         </is>
       </c>
       <c r="L10" s="13" t="inlineStr">
         <is>
-          <t>Eurasia Group 글로벌 커리어 포털 영문 CV/Cover Letter 제출</t>
+          <t>Palantir Global Careers Korea 포지션 지원</t>
         </is>
       </c>
       <c r="M10" s="11" t="inlineStr">
         <is>
-          <t>$80,000 - $120,000 USD (약 1억~1억 6,000만)</t>
+          <t>1억 2,000만 - 1억 8,000만+ (Base + Equity)</t>
         </is>
       </c>
       <c r="N10" s="13" t="inlineStr">
         <is>
-          <t>한반도 군사/지정학 리스크 평가, 다국적 기업 임원진 브리핑, 유려한 영문 리포팅.</t>
+          <t>국방/군사 고객 데이터 파이프라인 구축, 지휘통제(C4I) 및 작전 데이터 분석 모델 지원.</t>
         </is>
       </c>
       <c r="O10" s="13" t="inlineStr">
         <is>
-          <t>군사분계선(MDL)과 비물리적 분쟁을 실시간 다루는 현장 인텔리전스 분석력.</t>
+          <t>미8군/연합사 군사 교리 및 정전협정 데이터 실무 이해 + 파이썬 파이프라인 엔지니어링 역량 결합.</t>
         </is>
       </c>
       <c r="P10" s="10" t="n">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>현대차-GPO-2026</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>글로벌 정책전략실 (Global Public Policy) Specialist</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>과장급 (경력 3년~7년+)</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>현대자동차그룹 (Hyundai Motor Group)</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>서울 서초구 양재동 본사</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>대기업 글로벌전략</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>D-21</t>
-        </is>
-      </c>
-      <c r="K11" s="8" t="inlineStr">
-        <is>
-          <t>https://talent.hyundai.com/</t>
-        </is>
-      </c>
-      <c r="L11" s="9" t="inlineStr">
-        <is>
-          <t>현대자동차그룹 채용 포털 온라인 접수</t>
-        </is>
-      </c>
-      <c r="M11" s="7" t="inlineStr">
-        <is>
-          <t>7,500만 - 1억 1,000만+ (성과급 별도)</t>
-        </is>
-      </c>
-      <c r="N11" s="9" t="inlineStr">
-        <is>
-          <t>지정학적 통상 이슈 모니터링, 미국 정계/군/방산 정책 네트워크 대응, 영문 전략 보고서 작성.</t>
-        </is>
-      </c>
-      <c r="O11" s="9" t="inlineStr">
-        <is>
-          <t>정치외교학 학위 + 한미 안보 관계 실무 이해 + 미군 지휘부 네트워크 감각.</t>
-        </is>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>92</v>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Anduril-APAC-01</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>International Business Development (Korea Defense &amp; Autonomous Systems)</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Senior Manager / Director</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>Anduril Industries APAC (안두릴 코리아 사업단)</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
+          <t>서울 / 싱가포르 하이브리드</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>방산테크 &amp; CTI</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
+          <t>채용시 마감 (수시)</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="inlineStr">
+        <is>
+          <t>상시채용</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>https://www.anduril.com/careers/</t>
+        </is>
+      </c>
+      <c r="L11" s="17" t="inlineStr">
+        <is>
+          <t>Anduril 공식 채용 포털 지원</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>1억 3,000만 - 2억+ (Stock Options 포함)</t>
+        </is>
+      </c>
+      <c r="N11" s="17" t="inlineStr">
+        <is>
+          <t>자율 무기 체계(Lattice OS, 다이빙 DIVE-LD) 군 및 방위사업청 사업 제안, 한미 연합 작전 요구조건 조율.</t>
+        </is>
+      </c>
+      <c r="O11" s="17" t="inlineStr">
+        <is>
+          <t>UNCMAC 군사 번역 및 USFK J4 지정 통역관 출신. 군 지휘부 커뮤니케이션 완벽 소화.</t>
+        </is>
+      </c>
+      <c r="P11" s="14" t="n">
+        <v>97</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
@@ -1415,156 +1432,156 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>삼성전자-GPA-2026</t>
+          <t>한화에어로-글로벌전략</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>글로벌대외협력실 (GPA) 지정학 리스크 분석가</t>
+          <t>해외방산사업 글로벌 전략 기획자 (수출계약 및 절충교역)</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Professional (경력 4년+)</t>
+          <t>과장/차장급 (경력 5년+)</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>삼성전자 DS/DX 글로벌대외협력실</t>
+          <t>한화에어로스페이스 (Hanwha Aerospace)</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>서울 서초사옥 / 수원</t>
+          <t>서울 중구 청계천로 본사 / 창원</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>대기업 글로벌전략</t>
+          <t>방산테크 &amp; CTI</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="I12" s="10" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="J12" s="10" t="inlineStr">
         <is>
-          <t>D-16</t>
+          <t>D-28</t>
         </is>
       </c>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>https://www.samsungcareers.com</t>
+          <t>https://www.hanwhain.com</t>
         </is>
       </c>
       <c r="L12" s="13" t="inlineStr">
         <is>
-          <t>삼성채용 홈페이지 온라인 접수</t>
+          <t>한화인 온라인 채용 사이트 지원</t>
         </is>
       </c>
       <c r="M12" s="11" t="inlineStr">
         <is>
-          <t>8,000만 - 1억 2,000만+ (OPI/TAI 별도)</t>
+          <t>7,500만 - 1억 1,000만+ (성과급 별도)</t>
         </is>
       </c>
       <c r="N12" s="13" t="inlineStr">
         <is>
-          <t>미중 전략 경쟁 및 글로벌 공급망 안보 리스크 분석, 정부/의회 정책 대응 전략 수립.</t>
+          <t>해외 군 및 방산 획득 기관과의 수출 협상, 정부 대 정부(G2G) 방산 통상 조율, 영문 제안서 총괄.</t>
         </is>
       </c>
       <c r="O12" s="13" t="inlineStr">
         <is>
-          <t>국제정치학적 구조 분석 역량과 군사안보 데이터 분석 자동화 파이프라인 보유.</t>
+          <t>정치외교학 배경의 국가 간 무기 체계 획득 이해도 + 군사 영어 의전/협상 실전력.</t>
         </is>
       </c>
       <c r="P12" s="10" t="n">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Palantir-DS-Seoul</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Deployment Strategist (Palantir Korea)</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Senior / Lead Strategist</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>Palantir Technologies Korea</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>서울 강남구 (파르나스타워)</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>LIG넥스원-해외사업</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>해외사업본부 미국/APAC 방산 통상 및 프로젝트 관리</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>선임/책임연구원 (경력 4년+)</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>LIG넥스원 (LIG Nex1)</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>경기 성남시 판교 R&amp;D센터</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>방산테크 &amp; CTI</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>채용시 마감 (수시)</t>
-        </is>
-      </c>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>상시채용</t>
-        </is>
-      </c>
-      <c r="K13" s="8" t="inlineStr">
-        <is>
-          <t>https://www.palantir.com/careers/</t>
-        </is>
-      </c>
-      <c r="L13" s="9" t="inlineStr">
-        <is>
-          <t>Palantir 글로벌 커리어 사이트 영문 지원</t>
-        </is>
-      </c>
-      <c r="M13" s="7" t="inlineStr">
-        <is>
-          <t>1억 2,000만 - 1억 8,000만+ (Base + Equity)</t>
-        </is>
-      </c>
-      <c r="N13" s="9" t="inlineStr">
-        <is>
-          <t>국방/공공/대기업 대상 파운드리(Foundry) &amp; AIP 솔루션 도입 전략 수립, 복합 조직 워크플로우 재설계.</t>
-        </is>
-      </c>
-      <c r="O13" s="9" t="inlineStr">
-        <is>
-          <t>미 국방부/주한미군 데이터 체계 이해 + 파이썬 기반 데이터 파이프라인 자동화 아키텍처 역량.</t>
-        </is>
-      </c>
-      <c r="P13" s="6" t="n">
-        <v>96</v>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>D-25</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>https://lignex1.recruiter.co.kr</t>
+        </is>
+      </c>
+      <c r="L13" s="17" t="inlineStr">
+        <is>
+          <t>LIG넥스원 채용 포털 접수</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>7,000만 - 1억+ (성과급 별도)</t>
+        </is>
+      </c>
+      <c r="N13" s="17" t="inlineStr">
+        <is>
+          <t>미국 국방부 FCT(해외비교시험평가) 사업 대응, 비궁/신궁 등 유도무기 수출 계약 지원.</t>
+        </is>
+      </c>
+      <c r="O13" s="17" t="inlineStr">
+        <is>
+          <t>미군 지휘 행정 절차와 군사 작전 용어 완벽 숙지. 미국 국방 관계자 회의 조율 탁월.</t>
+        </is>
+      </c>
+      <c r="P13" s="14" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
@@ -1575,27 +1592,27 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>S2W-Threat-Analyst</t>
+          <t>S2W-Threat-Intel</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>사이버 위협 분석가 (Cyber Threat Intelligence / CTI Lead)</t>
+          <t>DarkWeb CTI Senior Threat Intelligence Analyst</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Senior Threat Analyst (경력 3년+)</t>
+          <t>시니어 분석가 (경력 3년+)</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>S2W (에스투더블유)</t>
+          <t>에스투더블유 (S2W Inc.)</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>경기 성남 판교 본사</t>
+          <t>경기 성남 판교 / 서울</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
@@ -1605,7 +1622,7 @@
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
@@ -1620,12 +1637,12 @@
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>https://www.wanted.co.kr/company/12717</t>
+          <t>https://s2w.inc/ko/careers</t>
         </is>
       </c>
       <c r="L14" s="13" t="inlineStr">
         <is>
-          <t>원티드 또는 S2W 공식 채용페이지 온라인 지원</t>
+          <t>S2W 공식 홈페이지 및 원티드 접수</t>
         </is>
       </c>
       <c r="M14" s="11" t="inlineStr">
@@ -1640,7 +1657,7 @@
       </c>
       <c r="O14" s="13" t="inlineStr">
         <is>
-          <t>정치외교학 배경과 《초한》 비물리전 시뮬레이션 기획으로 국가 행위자 인센티브 구조 분석 탁월.</t>
+          <t>정치외교학 배경과 비물리전 시뮬레이션 기획으로 국가 행위자 인센티브 구조 분석 탁월.</t>
         </is>
       </c>
       <c r="P14" s="10" t="n">
@@ -1648,82 +1665,82 @@
       </c>
     </row>
     <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>Nearthlab-Defense-BD</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>방산사업개발 리드 (Defense Business Development Lead)</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>팀장/리드급 (경력 5년+)</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>니어스랩 (Nearthlab)</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="14" t="inlineStr">
         <is>
           <t>서울 강남구 역삼동</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>방산테크 &amp; CTI</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="14" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I15" s="14" t="inlineStr">
         <is>
           <t>채용시 마감 (수시)</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="J15" s="14" t="inlineStr">
         <is>
           <t>상시채용</t>
         </is>
       </c>
-      <c r="K15" s="8" t="inlineStr">
+      <c r="K15" s="16" t="inlineStr">
         <is>
           <t>https://www.wanted.co.kr/company/3697</t>
         </is>
       </c>
-      <c r="L15" s="9" t="inlineStr">
+      <c r="L15" s="17" t="inlineStr">
         <is>
           <t>원티드 또는 니어스랩 채용포털 접수</t>
         </is>
       </c>
-      <c r="M15" s="7" t="inlineStr">
+      <c r="M15" s="15" t="inlineStr">
         <is>
           <t>7,000만 - 1억 1,000만+ (인센티브 별도)</t>
         </is>
       </c>
-      <c r="N15" s="9" t="inlineStr">
+      <c r="N15" s="17" t="inlineStr">
         <is>
           <t>자율비행 드론 기반 국방/정찰/감시 솔루션 군 및 방산기관 납품 사업 개발, 제안서 작성.</t>
         </is>
       </c>
-      <c r="O15" s="9" t="inlineStr">
+      <c r="O15" s="17" t="inlineStr">
         <is>
           <t>한미 연합 지휘구조 이해 및 군사 기술 문서화/브리핑 역량.</t>
         </is>
       </c>
-      <c r="P15" s="6" t="n">
+      <c r="P15" s="14" t="n">
         <v>93</v>
       </c>
     </row>
@@ -1800,7 +1817,7 @@
       </c>
       <c r="O16" s="13" t="inlineStr">
         <is>
-          <t>UNCMAC 보안 프로토콜 및 Antigravity 파이썬 파이프라인 엔지니어링 실무 융합.</t>
+          <t>UNCMAC 보안 프로토콜 및 데이터 자동화 파이프라인 엔지니어링 실무 융합.</t>
         </is>
       </c>
       <c r="P16" s="10" t="n">
@@ -1808,82 +1825,82 @@
       </c>
     </row>
     <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>AWS-WWPS-SA-01</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <t>Solutions Architect (Public Sector &amp; Defense)</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="15" t="inlineStr">
         <is>
           <t>L5 / Senior SA</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="15" t="inlineStr">
         <is>
           <t>Amazon Web Services Korea (AWS WWPS)</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>서울 강남구 역삼동 (센터필드)</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="14" t="inlineStr">
         <is>
           <t>글로벌 빅테크/IT</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="14" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="I17" s="14" t="inlineStr">
         <is>
           <t>채용시 마감 (수시)</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J17" s="14" t="inlineStr">
         <is>
           <t>상시채용</t>
         </is>
       </c>
-      <c r="K17" s="8" t="inlineStr">
+      <c r="K17" s="16" t="inlineStr">
         <is>
           <t>https://www.amazon.jobs/en/locations/seoul-south-korea</t>
         </is>
       </c>
-      <c r="L17" s="9" t="inlineStr">
+      <c r="L17" s="17" t="inlineStr">
         <is>
           <t>Amazon Jobs 공식 포털 지원</t>
         </is>
       </c>
-      <c r="M17" s="7" t="inlineStr">
+      <c r="M17" s="15" t="inlineStr">
         <is>
           <t>1억 1,000만 - 1억 6,000만+ (Base + RSU)</t>
         </is>
       </c>
-      <c r="N17" s="9" t="inlineStr">
+      <c r="N17" s="17" t="inlineStr">
         <is>
           <t>정부/공공/국방 고객 대상 클라우드 아키텍처 컨설팅, 망분리 및 보안 인증 대응.</t>
         </is>
       </c>
-      <c r="O17" s="9" t="inlineStr">
+      <c r="O17" s="17" t="inlineStr">
         <is>
           <t>국방 조직의 보안 요구조건과 지휘 통신 워크플로우에 대한 현장 경험.</t>
         </is>
       </c>
-      <c r="P17" s="6" t="n">
+      <c r="P17" s="14" t="n">
         <v>91</v>
       </c>
     </row>
@@ -1968,89 +1985,249 @@
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>KRAFTON-Narrative-01</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="15" t="inlineStr">
         <is>
           <t>시니어 내러티브 디자이너 (Narrative Lead / 정치스릴러)</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>시니어급 (경력 3년~5년+)</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>크래프톤 (KRAFTON)</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="14" t="inlineStr">
         <is>
           <t>서울 강남 / 경기 성남 판교</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G19" s="14" t="inlineStr">
         <is>
           <t>게임 내러티브 / AI 시스템</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="14" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I19" s="14" t="inlineStr">
         <is>
           <t>채용시 마감 (수시)</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J19" s="14" t="inlineStr">
         <is>
           <t>상시채용</t>
         </is>
       </c>
-      <c r="K19" s="8" t="inlineStr">
+      <c r="K19" s="16" t="inlineStr">
         <is>
           <t>https://krafton.com/careers/</t>
         </is>
       </c>
-      <c r="L19" s="9" t="inlineStr">
+      <c r="L19" s="17" t="inlineStr">
         <is>
           <t>크래프톤 공식 채용 사이트 온라인 접수</t>
         </is>
       </c>
-      <c r="M19" s="7" t="inlineStr">
+      <c r="M19" s="15" t="inlineStr">
         <is>
           <t>6,500만 - 9,500만+ + 인센티브</t>
         </is>
       </c>
-      <c r="N19" s="9" t="inlineStr">
+      <c r="N19" s="17" t="inlineStr">
         <is>
           <t>치밀한 진영 갈등 및 현실감 넘치는 세계관 설정, 대사 스크립트 작성.</t>
         </is>
       </c>
-      <c r="O19" s="9" t="inlineStr">
+      <c r="O19" s="17" t="inlineStr">
         <is>
           <t>실제 정치·안보 분석 데이터 기반의 하이브리드전 비주얼 노벨 《초한》 제작 포트폴리오 보유.</t>
         </is>
       </c>
-      <c r="P19" s="6" t="n">
+      <c r="P19" s="14" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>🔍 상시모니터링</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>LINKEDIN-FEED-DEFENSE</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>LinkedIn 실시간 피드: Defense Tech &amp; Security Policy Korea</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Senior / Lead / Specialist</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>LinkedIn Korea Job Search Network</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Seoul / Remote</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>커리어포털 상시피드</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>실시간 업데이트</t>
+        </is>
+      </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>상시감시</t>
+        </is>
+      </c>
+      <c r="K20" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=defense%20policy%20korea</t>
+        </is>
+      </c>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>LinkedIn 공고별 직접 지원</t>
+        </is>
+      </c>
+      <c r="M20" s="11" t="inlineStr">
+        <is>
+          <t>포지션별 상이</t>
+        </is>
+      </c>
+      <c r="N20" s="13" t="inlineStr">
+        <is>
+          <t>방산, 안보 정책, 정부 대관, 한미 안보 협력 키워드 실시간 공고 피드.</t>
+        </is>
+      </c>
+      <c r="O20" s="13" t="inlineStr">
+        <is>
+          <t>글로벌 방산 및 보안 기업 상시 헤드헌팅 네트워크 직결.</t>
+        </is>
+      </c>
+      <c r="P20" s="10" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>🔍 상시모니터링</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>WANTED-FEED-DEFENSE</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>원티드 실시간 피드: 국방 / 방산 / 통역 / 대외협력 전문직</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>경력 3년 이상 전문직</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>Wanted Lab (원티드)</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>대한민국 전역</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>커리어포털 상시피드</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>실시간 업데이트</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="inlineStr">
+        <is>
+          <t>상시감시</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>https://www.wanted.co.kr/search?query=%EA%B5%AD%EB%B0%A9</t>
+        </is>
+      </c>
+      <c r="L21" s="17" t="inlineStr">
+        <is>
+          <t>원티드 플랫폼 내 원클릭 지원</t>
+        </is>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>포지션별 상이</t>
+        </is>
+      </c>
+      <c r="N21" s="17" t="inlineStr">
+        <is>
+          <t>원티드 등록 국내 방산 및 기술 스타트업 채용 실시간 트래킹.</t>
+        </is>
+      </c>
+      <c r="O21" s="17" t="inlineStr">
+        <is>
+          <t>신속한 채용 지원 및 합격 보상금 연계.</t>
+        </is>
+      </c>
+      <c r="P21" s="14" t="n">
         <v>90</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="A2:A500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"🟢 진행중,⏳ 순환 대기,🔍 상시모니터링,📌 관심등록,📝 지원서작성,🚀 접수완료"</formula1>
+      <formula1>"🟢 실시간 접수중,🟢 진행중,🔍 1일단위 감시중,🔍 상시모니터링,📌 관심등록,📝 지원서작성,🚀 접수완료"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -2072,6 +2249,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Optimize for iPhone Safari Web App and remove all text cutoffs
</commit_message>
<xml_diff>
--- a/Career_Opportunity_Master.xlsx
+++ b/Career_Opportunity_Master.xlsx
@@ -624,7 +624,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>🟢 실시간 접수중</t>
@@ -704,7 +704,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>🔍 1일단위 감시중</t>
@@ -784,7 +784,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -864,7 +864,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="48" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -944,7 +944,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1024,7 +1024,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1104,7 +1104,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1184,7 +1184,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
+    <row r="9" ht="48" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1264,7 +1264,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
+    <row r="10" ht="48" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1344,7 +1344,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
+    <row r="11" ht="54" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1424,7 +1424,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="12" ht="42" customHeight="1">
+    <row r="12" ht="48" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1504,7 +1504,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="13" ht="42" customHeight="1">
+    <row r="13" ht="48" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1584,7 +1584,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="14" ht="42" customHeight="1">
+    <row r="14" ht="48" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1664,7 +1664,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="15" ht="42" customHeight="1">
+    <row r="15" ht="48" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1744,7 +1744,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1">
+    <row r="16" ht="48" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1824,7 +1824,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="17" ht="42" customHeight="1">
+    <row r="17" ht="48" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1904,7 +1904,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1">
+    <row r="18" ht="48" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -1984,7 +1984,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="19" ht="42" customHeight="1">
+    <row r="19" ht="48" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
           <t>🟢 진행중</t>
@@ -2064,7 +2064,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="20" ht="42" customHeight="1">
+    <row r="20" ht="48" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
           <t>🔍 상시모니터링</t>
@@ -2144,7 +2144,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="21" ht="42" customHeight="1">
+    <row r="21" ht="48" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
           <t>🔍 상시모니터링</t>

</xml_diff>